<commit_message>
feat(currency-wars): G12-P3-B5 author complete workbooks
</commit_message>
<xml_diff>
--- a/config/currency-wars-generated/templates/CurrencyWarsBindings.xlsx
+++ b/config/currency-wars-generated/templates/CurrencyWarsBindings.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="188">
   <si>
     <t>@table</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>length=2..32767</t>
+  </si>
+  <si>
+    <t>length=0..32767</t>
   </si>
   <si>
     <t>#desc</t>
@@ -1325,18 +1328,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1388,7 +1391,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1412,7 +1415,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -1459,13 +1462,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -1512,13 +1515,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -1671,18 +1674,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1733,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1757,7 +1760,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -1804,16 +1807,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -1860,16 +1863,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -2028,21 +2031,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2096,7 +2099,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2120,7 +2123,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -2167,13 +2170,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -2220,13 +2223,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -2379,18 +2382,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2441,7 +2444,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2465,7 +2468,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -2512,22 +2515,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -2574,22 +2577,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -2760,27 +2763,27 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2834,7 +2837,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2858,7 +2861,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -2905,19 +2908,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -2964,19 +2967,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -3141,24 +3144,24 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3211,7 +3214,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3235,7 +3238,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -3282,16 +3285,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -3338,16 +3341,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -3506,21 +3509,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3572,7 +3575,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3596,7 +3599,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -3643,13 +3646,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -3696,13 +3699,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -3855,18 +3858,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3921,7 +3924,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3945,7 +3948,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -3992,16 +3995,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -4048,16 +4051,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -4216,21 +4219,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4283,7 +4286,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4307,7 +4310,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -4354,19 +4357,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -4413,19 +4416,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -4590,24 +4593,24 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4660,7 +4663,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4684,7 +4687,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -4731,13 +4734,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -4784,13 +4787,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -4943,18 +4946,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -5005,7 +5008,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5029,7 +5032,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -5079,13 +5082,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -5135,13 +5138,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -5300,21 +5303,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -5370,7 +5373,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5394,7 +5397,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -5441,16 +5444,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -5497,16 +5500,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -5665,21 +5668,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -5731,7 +5734,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5755,7 +5758,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -5802,13 +5805,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -5855,13 +5858,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -6014,18 +6017,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -6077,7 +6080,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6101,7 +6104,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -6148,13 +6151,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -6201,13 +6204,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -6360,18 +6363,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -6423,7 +6426,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6447,7 +6450,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -6494,13 +6497,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -6547,13 +6550,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -6706,18 +6709,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -6771,7 +6774,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6795,7 +6798,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -6842,13 +6845,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -6895,13 +6898,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -7054,18 +7057,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -7116,7 +7119,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7140,7 +7143,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -7187,16 +7190,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7243,16 +7246,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7411,21 +7414,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -7479,7 +7482,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7503,7 +7506,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -7550,16 +7553,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7606,16 +7609,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7774,21 +7777,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -7842,7 +7845,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7866,7 +7869,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -7913,16 +7916,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7969,16 +7972,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -8137,21 +8140,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -8204,7 +8207,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8228,7 +8231,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -8275,13 +8278,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -8328,13 +8331,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -8487,18 +8490,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -8552,7 +8555,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8576,7 +8579,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -8623,16 +8626,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -8679,16 +8682,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -8847,21 +8850,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -8913,7 +8916,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8937,7 +8940,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -8984,16 +8987,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -9040,16 +9043,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -9208,21 +9211,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -9276,7 +9279,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9300,7 +9303,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -9347,16 +9350,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -9403,16 +9406,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -9571,21 +9574,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -9637,7 +9640,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9661,7 +9664,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -9708,19 +9711,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -9767,19 +9770,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -9944,24 +9947,24 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -10017,7 +10020,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10041,7 +10044,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -10088,16 +10091,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -10144,16 +10147,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -10312,21 +10315,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -10381,7 +10384,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10405,7 +10408,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -10452,13 +10455,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -10505,13 +10508,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -10664,18 +10667,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -10728,7 +10731,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10752,7 +10755,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -10799,16 +10802,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -10855,16 +10858,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -11023,21 +11026,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -11091,7 +11094,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -11115,7 +11118,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -11162,13 +11165,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -11215,13 +11218,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -11374,18 +11377,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -11439,7 +11442,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -11463,7 +11466,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -11510,16 +11513,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -11566,16 +11569,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -11734,21 +11737,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -11803,7 +11806,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -11827,7 +11830,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -11874,13 +11877,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -11927,13 +11930,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -12086,18 +12089,18 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -12149,7 +12152,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12173,7 +12176,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -12220,16 +12223,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -12276,16 +12279,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -12444,21 +12447,21 @@
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>

</xml_diff>

<commit_message>
feat(currency-wars): implement complete runtime
</commit_message>
<xml_diff>
--- a/config/currency-wars-generated/templates/CurrencyWarsBindings.xlsx
+++ b/config/currency-wars-generated/templates/CurrencyWarsBindings.xlsx
@@ -34,18 +34,24 @@
     <sheet name="Currencies" sheetId="25" r:id="rId25"/>
     <sheet name="ShopServices" sheetId="26" r:id="rId26"/>
     <sheet name="ServiceOfferRules" sheetId="27" r:id="rId27"/>
-    <sheet name="EncounterSourceObligations" sheetId="28" r:id="rId28"/>
-    <sheet name="EncounterGroups" sheetId="29" r:id="rId29"/>
-    <sheet name="EncounterWaves" sheetId="30" r:id="rId30"/>
-    <sheet name="EnemySlots" sheetId="31" r:id="rId31"/>
-    <sheet name="BossPools" sheetId="32" r:id="rId32"/>
+    <sheet name="RewardDefinitions" sheetId="28" r:id="rId28"/>
+    <sheet name="RewardPools" sheetId="29" r:id="rId29"/>
+    <sheet name="EquipmentRecipes" sheetId="30" r:id="rId30"/>
+    <sheet name="EquipmentUpgrades" sheetId="31" r:id="rId31"/>
+    <sheet name="ForgeServices" sheetId="32" r:id="rId32"/>
+    <sheet name="ServiceConstants" sheetId="33" r:id="rId33"/>
+    <sheet name="EncounterSourceObligations" sheetId="34" r:id="rId34"/>
+    <sheet name="EncounterGroups" sheetId="35" r:id="rId35"/>
+    <sheet name="EncounterWaves" sheetId="36" r:id="rId36"/>
+    <sheet name="EnemySlots" sheetId="37" r:id="rId37"/>
+    <sheet name="BossPools" sheetId="38" r:id="rId38"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3858" uniqueCount="224">
   <si>
     <t>@table</t>
   </si>
@@ -65,16 +71,16 @@
     <t>id</t>
   </si>
   <si>
-    <t>@scope</t>
-  </si>
-  <si>
-    <t>all</t>
+    <t>@groups</t>
+  </si>
+  <si>
+    <t>common</t>
   </si>
   <si>
     <t>@schema</t>
   </si>
   <si>
-    <t>d72d68afe6525021</t>
+    <t>5b8fd72e699d2ba9</t>
   </si>
   <si>
     <t>#name</t>
@@ -140,7 +146,7 @@
     <t>optional&lt;string&gt;</t>
   </si>
   <si>
-    <t>#scope</t>
+    <t>#groups</t>
   </si>
   <si>
     <t>#input</t>
@@ -158,7 +164,7 @@
     <t>CurrencyWarsBlessings</t>
   </si>
   <si>
-    <t>2bf089c16390ec19</t>
+    <t>b7ca0d9b3e214f4f</t>
   </si>
   <si>
     <t>category</t>
@@ -173,7 +179,7 @@
     <t>CurrencyWarsBlessingLevels</t>
   </si>
   <si>
-    <t>cb573c280b8687a8</t>
+    <t>cc45495e82c4c3f2</t>
   </si>
   <si>
     <t>blessing_id</t>
@@ -188,7 +194,7 @@
     <t>CurrencyWarsBlessingGroups</t>
   </si>
   <si>
-    <t>927ab95c5008ee42</t>
+    <t>ef9bd45ae1d503e6</t>
   </si>
   <si>
     <t>candidate_ids</t>
@@ -203,7 +209,7 @@
     <t>CurrencyWarsFormulas</t>
   </si>
   <si>
-    <t>1d90bf907d9429dd</t>
+    <t>8da9986446e387e3</t>
   </si>
   <si>
     <t>formula_kind</t>
@@ -218,7 +224,7 @@
     <t>CurrencyWarsFormulaDisplays</t>
   </si>
   <si>
-    <t>8f258b1787f1cfed</t>
+    <t>f998afba1ac8db0d</t>
   </si>
   <si>
     <t>formula_id</t>
@@ -233,7 +239,7 @@
     <t>CurrencyWarsFormulaRandomizers</t>
   </si>
   <si>
-    <t>1281c77f1a6bdb8b</t>
+    <t>74526d921bb0cf5f</t>
   </si>
   <si>
     <t>reroll_rule</t>
@@ -245,7 +251,7 @@
     <t>CurrencyWarsFormulaRecipes</t>
   </si>
   <si>
-    <t>94bb8c1c5aaadb05</t>
+    <t>586021e11824a4a1</t>
   </si>
   <si>
     <t>required_path_counts</t>
@@ -260,7 +266,7 @@
     <t>CurrencyWarsFormulaContributions</t>
   </si>
   <si>
-    <t>ecb9a96347b0be01</t>
+    <t>1dd6b81799952351</t>
   </si>
   <si>
     <t>source_state</t>
@@ -275,7 +281,7 @@
     <t>CurrencyWarsCurios</t>
   </si>
   <si>
-    <t>d640865fbde07b9f</t>
+    <t>d0e80678e3c6fcf3</t>
   </si>
   <si>
     <t>state_ids</t>
@@ -287,7 +293,7 @@
     <t>CurrencyWarsCurioStates</t>
   </si>
   <si>
-    <t>0b1d9a229af21efd</t>
+    <t>4617a1e5a50eb71d</t>
   </si>
   <si>
     <t>curio_id</t>
@@ -302,7 +308,7 @@
     <t>CurrencyWarsCurioGroups</t>
   </si>
   <si>
-    <t>593277e04e54360f</t>
+    <t>7e60dca72808a335</t>
   </si>
   <si>
     <t>candidate_state_ids</t>
@@ -317,7 +323,7 @@
     <t>CurrencyWarsCurioLifecycleRules</t>
   </si>
   <si>
-    <t>7d9435f5fafb8d69</t>
+    <t>8d5da4d7bb3622b9</t>
   </si>
   <si>
     <t>activation</t>
@@ -335,7 +341,7 @@
     <t>CurrencyWarsHexStates</t>
   </si>
   <si>
-    <t>685f7268e7ff3ab0</t>
+    <t>e2ab5547871cda30</t>
   </si>
   <si>
     <t>hex_id</t>
@@ -347,7 +353,7 @@
     <t>CurrencyWarsHexEligibility</t>
   </si>
   <si>
-    <t>d50276af9fadd16b</t>
+    <t>fb40df7a69493941</t>
   </si>
   <si>
     <t>subject_id</t>
@@ -356,7 +362,7 @@
     <t>CurrencyWarsOccurrences</t>
   </si>
   <si>
-    <t>7b09b892c7dbf2db</t>
+    <t>0cf02282dd5dfc4b</t>
   </si>
   <si>
     <t>variant_ids</t>
@@ -371,7 +377,7 @@
     <t>CurrencyWarsOccurrenceVariants</t>
   </si>
   <si>
-    <t>554780e7f9a9999c</t>
+    <t>e64e0a9565084762</t>
   </si>
   <si>
     <t>occurrence_id</t>
@@ -386,7 +392,7 @@
     <t>CurrencyWarsOccurrenceChoices</t>
   </si>
   <si>
-    <t>6e60116838a5d021</t>
+    <t>b0c4a1de44267697</t>
   </si>
   <si>
     <t>variant_id</t>
@@ -407,7 +413,7 @@
     <t>CurrencyWarsWorkbenches</t>
   </si>
   <si>
-    <t>fb3fbf9200a56708</t>
+    <t>44847cbc0d243f9e</t>
   </si>
   <si>
     <t>function_ids</t>
@@ -422,7 +428,7 @@
     <t>CurrencyWarsWorkbenchFunctions</t>
   </si>
   <si>
-    <t>b975ac924e1ff91f</t>
+    <t>8c577e983dc47fef</t>
   </si>
   <si>
     <t>function_type</t>
@@ -440,7 +446,7 @@
     <t>CurrencyWarsGambleGroups</t>
   </si>
   <si>
-    <t>07725784bee85973</t>
+    <t>932d8bbcd2a4c75d</t>
   </si>
   <si>
     <t>group_type</t>
@@ -455,7 +461,7 @@
     <t>CurrencyWarsGambleUnits</t>
   </si>
   <si>
-    <t>8095421ede159850</t>
+    <t>bac91f9877ae08ee</t>
   </si>
   <si>
     <t>unit_type</t>
@@ -467,7 +473,7 @@
     <t>CurrencyWarsCurseChests</t>
   </si>
   <si>
-    <t>9491408a8b579083</t>
+    <t>e921b5dc3dc09ffb</t>
   </si>
   <si>
     <t>chest_type</t>
@@ -479,7 +485,7 @@
     <t>CurrencyWarsAdventureOutcomes</t>
   </si>
   <si>
-    <t>3d28053e71fcd2cd</t>
+    <t>1b7c4c37d3e9304b</t>
   </si>
   <si>
     <t>adventure_type</t>
@@ -494,7 +500,7 @@
     <t>CurrencyWarsCurrencies</t>
   </si>
   <si>
-    <t>e6d928c74dbdc14d</t>
+    <t>d7f0d02cae2b4005</t>
   </si>
   <si>
     <t>gain_rules</t>
@@ -509,7 +515,7 @@
     <t>CurrencyWarsShopServices</t>
   </si>
   <si>
-    <t>516f363c40d0cdba</t>
+    <t>a42a45c22cba83fc</t>
   </si>
   <si>
     <t>service_kind</t>
@@ -524,16 +530,103 @@
     <t>CurrencyWarsServiceOfferRules</t>
   </si>
   <si>
-    <t>26f4d8f5f89109ff</t>
+    <t>78eb8d8c14782e69</t>
   </si>
   <si>
     <t>service_id</t>
   </si>
   <si>
+    <t>CurrencyWarsRewardDefinitions</t>
+  </si>
+  <si>
+    <t>a927b34e8b00f07a</t>
+  </si>
+  <si>
+    <t>source_id</t>
+  </si>
+  <si>
+    <t>operation_kind</t>
+  </si>
+  <si>
+    <t>budget_cost</t>
+  </si>
+  <si>
+    <t>scalar_parameter</t>
+  </si>
+  <si>
+    <t>CurrencyWarsRewardPools</t>
+  </si>
+  <si>
+    <t>7a653f13671dd990</t>
+  </si>
+  <si>
+    <t>total_value</t>
+  </si>
+  <si>
+    <t>candidate_bonus_ids</t>
+  </si>
+  <si>
+    <t>candidate_maximums</t>
+  </si>
+  <si>
+    <t>candidate_weights</t>
+  </si>
+  <si>
+    <t>CurrencyWarsEquipmentRecipes</t>
+  </si>
+  <si>
+    <t>a29c643eddafed94</t>
+  </si>
+  <si>
+    <t>season_id</t>
+  </si>
+  <si>
+    <t>output_equipment_id</t>
+  </si>
+  <si>
+    <t>input_equipment_ids</t>
+  </si>
+  <si>
+    <t>CurrencyWarsEquipmentUpgrades</t>
+  </si>
+  <si>
+    <t>0cb7adf509778482</t>
+  </si>
+  <si>
+    <t>source_equipment_id</t>
+  </si>
+  <si>
+    <t>CurrencyWarsForgeServices</t>
+  </si>
+  <si>
+    <t>6ba4a7be88eeb8c4</t>
+  </si>
+  <si>
+    <t>equipment_category</t>
+  </si>
+  <si>
+    <t>offer_count</t>
+  </si>
+  <si>
+    <t>target_kind</t>
+  </si>
+  <si>
+    <t>CurrencyWarsServiceConstants</t>
+  </si>
+  <si>
+    <t>d5f184be2b541ada</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>consumer_policy</t>
+  </si>
+  <si>
     <t>CurrencyWarsEncounterSourceObligations</t>
   </si>
   <si>
-    <t>2891e8bcab3c5ee5</t>
+    <t>d78af67b1076bd22</t>
   </si>
   <si>
     <t>parent_kind</t>
@@ -545,10 +638,22 @@
     <t>resolution_state</t>
   </si>
   <si>
+    <t>stage_id</t>
+  </si>
+  <si>
+    <t>camp_ids</t>
+  </si>
+  <si>
+    <t>stage_snapshot</t>
+  </si>
+  <si>
+    <t>replacement_condition</t>
+  </si>
+  <si>
     <t>CurrencyWarsEncounterGroups</t>
   </si>
   <si>
-    <t>638d0e3cc939b04c</t>
+    <t>870d547d7d0bccd5</t>
   </si>
   <si>
     <t>plane_id</t>
@@ -563,13 +668,22 @@
     <t>candidate_stage_ids</t>
   </si>
   <si>
+    <t>monster_ids</t>
+  </si>
+  <si>
+    <t>battle_area_ids</t>
+  </si>
+  <si>
+    <t>boss_battle_area_id</t>
+  </si>
+  <si>
+    <t>randomization</t>
+  </si>
+  <si>
     <t>CurrencyWarsEncounterWaves</t>
   </si>
   <si>
-    <t>33fbbe2edb83d1ae</t>
-  </si>
-  <si>
-    <t>stage_id</t>
+    <t>81930e1f85fa7a30</t>
   </si>
   <si>
     <t>wave_index</t>
@@ -584,7 +698,7 @@
     <t>CurrencyWarsEnemySlots</t>
   </si>
   <si>
-    <t>642a6c4046583923</t>
+    <t>6716a11a05671007</t>
   </si>
   <si>
     <t>wave_id</t>
@@ -599,10 +713,13 @@
     <t>ability_refs</t>
   </si>
   <si>
+    <t>shared_enemy_key</t>
+  </si>
+  <si>
     <t>CurrencyWarsBossPools</t>
   </si>
   <si>
-    <t>72428a8566d13104</t>
+    <t>746e4fac5c6861a3</t>
   </si>
   <si>
     <t>candidate_monster_ids</t>
@@ -8186,7 +8303,7 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -8198,10 +8315,10 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
+    <col min="15" max="19" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8233,7 +8350,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="24" customHeight="1">
+    <row r="2" spans="1:19" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -8283,10 +8400,16 @@
         <v>164</v>
       </c>
       <c r="Q2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="S2" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
@@ -8336,10 +8459,16 @@
         <v>164</v>
       </c>
       <c r="Q3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" s="5" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="4" spans="1:17">
+      <c r="S3" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4" s="4" t="s">
         <v>27</v>
       </c>
@@ -8391,8 +8520,14 @@
       <c r="Q4" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:17">
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
       <c r="A5" s="4" t="s">
         <v>31</v>
       </c>
@@ -8444,8 +8579,14 @@
       <c r="Q5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:17">
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
@@ -8497,370 +8638,14 @@
       <c r="Q6" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="42" customHeight="1">
-      <c r="A7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
-      <formula1>1</formula1>
-      <formula2>2147483647</formula2>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
-    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
-    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
-    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
-    <col min="18" max="18" width="19.7109375" style="5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="24" customHeight="1">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
-      <c r="A3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18">
-      <c r="A4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18">
-      <c r="A5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="R5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18">
-      <c r="A6" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>34</v>
-      </c>
       <c r="R6" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="S6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>35</v>
       </c>
@@ -8881,6 +8666,405 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="16" width="16.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="19.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="18.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="17.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -9269,7 +9453,8 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="18" width="16.7109375" style="5" customWidth="1"/>
+    <col min="15" max="16" width="16.7109375" style="5" customWidth="1"/>
+    <col min="17" max="18" width="19.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -9277,7 +9462,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9301,7 +9486,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -9348,7 +9533,7 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>175</v>
@@ -9404,7 +9589,7 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>175</v>
@@ -9619,6 +9804,336 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="16" width="19.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -9631,7 +10146,9 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="19" width="16.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="18.7109375" style="5" customWidth="1"/>
+    <col min="17" max="19" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -9639,7 +10156,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9663,7 +10180,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -9710,19 +10227,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>183</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -9769,19 +10286,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>183</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -9995,9 +10512,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -10009,17 +10526,15 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="16" width="16.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
-    <col min="18" max="18" width="16.7109375" style="5" customWidth="1"/>
+    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10043,10 +10558,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="24" customHeight="1">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -10090,19 +10605,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
@@ -10146,19 +10658,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="4" t="s">
         <v>27</v>
       </c>
@@ -10210,11 +10719,8 @@
       <c r="Q4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="R4" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18">
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="4" t="s">
         <v>31</v>
       </c>
@@ -10266,11 +10772,8 @@
       <c r="Q5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="R5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18">
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
@@ -10322,11 +10825,415 @@
       <c r="Q6" s="5" t="s">
         <v>34</v>
       </c>
+    </row>
+    <row r="7" spans="1:17" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="20" width="16.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="21.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="R6" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="S6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>35</v>
       </c>
@@ -10347,6 +11254,1592 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:V7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="19.7109375" style="5" customWidth="1"/>
+    <col min="19" max="20" width="16.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="19.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="18" width="16.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="20" width="16.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="16" width="16.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" style="5" customWidth="1"/>
+    <col min="19" max="20" width="19.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>